<commit_message>
Rebuild the import template: a column per photo, and a thumbnail
Semicolons in one cell are hard to fill in by hand and easy to get wrong.
Each photo now has its own column, photo_1 to photo_6 — the catalogue
averages 2.3 photos and peaks at 4, so six is headroom without a wall of
empty columns.

thumbnail is a separate image rather than a pointer at one of the photos:
the shop wants control over the single picture a customer sees while
browsing. Blank falls back to photo_1, so it is optional per product.

The field does not exist in the schema yet. Products has only the photos
array and the storefront uses photos[0] for the grid, so a thumbnail upload
field, a migration and a change to the grid components are all needed
before an import can run. Noted at the bottom of the README.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import/products-template.xlsx
+++ b/docs/import/products-template.xlsx
@@ -49,7 +49,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +64,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFD9D2"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,12 +89,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -466,30 +474,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="28" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="28" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -500,308 +514,366 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>photos</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+          <t>photo_1</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>photo_2</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>photo_3</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>photo_4</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>photo_5</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>photo_6</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>thumbnail</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>mrp</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>subCategory</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>occasions</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>countryOfOrigin</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>genericName</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>netQuantity</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>dimensions</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>finish</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>monthYearOfImport</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>featured</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>shortCaption</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>shortSticker</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Krishna with flute — Venugopala form</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Krishna with flute - Venugopala form</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>krishna-flute-01.jpg;krishna-flute-02.jpg</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
+          <t>krishna-flute-01.jpg</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>krishna-flute-02.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>krishna-flute-03.jpg</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>krishna-flute-thumb.jpg</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="n">
         <v>3950</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="J2" s="4" t="n">
         <v>4500</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="K2" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>pooja</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Brass Idols</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Brass Krishna standing with a flute, on a lotus base.</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>festival;wedding</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>Sri Balaji Handicrafts</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>Brass idol</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>1 piece</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>9 x 4 x 3 in</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>850 g</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>Antique brass</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>09/2026</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>The one everyone asks for</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>Bestseller</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Leather sling bag — tan</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Leather sling bag - tan</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>tan-sling-01.jpg;tan-sling-02.jpg;tan-sling-03.jpg</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
+          <t>tan-sling-01.jpg</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>tan-sling-02.jpg</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="n">
         <v>1299</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="J3" s="4" t="n">
         <v>1799</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="K3" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>bags</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Slings &amp; Crossbody</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Compact tan sling with an adjustable strap and two zip pockets.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>birthday;everyday</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>Hidesign Leathers</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>Sling bag</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>1 piece</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>10 x 7 x 3 in</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="U3" s="4" t="inlineStr">
         <is>
           <t>420 g</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="V3" s="4" t="inlineStr">
         <is>
           <t>Genuine leather</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="W3" s="4" t="inlineStr">
         <is>
           <t>08/2026</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr"/>
-      <c r="U3" s="3" t="inlineStr"/>
+      <c r="Z3" s="4" t="inlineStr"/>
+      <c r="AA3" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="One of the eight section codes — see the 'Section codes' sheet." promptTitle="Pick from the list" prompt="One of the eight section codes — see the 'Section codes' sheet." type="list">
+    <dataValidation sqref="L2:L2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="One of the eight section codes - see the 'Section codes' sheet." promptTitle="Pick from the list" prompt="One of the eight section codes - see the 'Section codes' sheet." type="list">
       <formula1>"decor,pooja,fashion,bags,shoes,watches,gifting,lifestyle"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="live = on the website. draft = held back. hidden = retired." promptTitle="Pick from the list" prompt="live = on the website. draft = held back. hidden = retired." type="list">
+    <dataValidation sqref="X2:X2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="live = on the website. draft = held back. hidden = retired." promptTitle="Pick from the list" prompt="live = on the website. draft = held back. hidden = retired." type="list">
       <formula1>"live,draft,hidden"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="yes puts it in the Shoppable Shorts rail. Keep this to a handful." promptTitle="Pick from the list" prompt="yes puts it in the Shoppable Shorts rail. Keep this to a handful." type="list">
+    <dataValidation sqref="Y2:Y2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="yes puts it in the Shoppable Shorts rail. Keep this to a handful." promptTitle="Pick from the list" prompt="yes puts it in the Shoppable Shorts rail. Keep this to a handful." type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -823,12 +895,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Code (use this)</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Section shown on the website</t>
         </is>
@@ -842,7 +914,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Home &amp; Décor</t>
+          <t>Home &amp; Decor</t>
         </is>
       </c>
     </row>
@@ -941,223 +1013,301 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="118" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>The One Roof — bulk product upload</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>The One Roof - bulk product upload</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
+      <c r="A2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>One row is one product. Fill in the Products sheet, put all the photos in ONE folder, send both.</t>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>One row is one product. Fill in the Products sheet, put ALL the images in ONE folder, send both.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Gold headers are required. Grey headers are optional — leave them blank if you don't have the information.</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Gold headers are required. Green is the thumbnail. Grey is optional - leave blank if you don't have it.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
+      <c r="A5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>PHOTOS — this is the part that goes wrong</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>PHOTOS - one per column</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Name every photo after its product, numbered:</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Put each photo's filename in its own column: photo_1, photo_2, and so on. Up to six.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      krishna-flute-01.jpg      &lt;- the first one shows in the shop grid, so pick the best</t>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Leave the rest blank. Most products need two or three.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      krishna-flute-02.jpg</t>
-        </is>
-      </c>
+      <c r="A9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Then list them in the photos column, separated by semicolons, best first:</t>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      photo_1   krishna-flute-01.jpg</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      krishna-flute-01.jpg;krishna-flute-02.jpg</t>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      photo_2   krishna-flute-02.jpg</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      photo_3   krishna-flute-03.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      • No spaces in filenames. Use hyphens.</t>
-        </is>
-      </c>
+      <c r="A13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      • Every filename must exist in the folder, spelled identically.</t>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>These are the pictures on the product's own page, in the order you list them.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Krishna-Flute-01.JPG and krishna-flute-01.jpg are different files.</t>
-        </is>
-      </c>
+      <c r="A15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">      • Send the photos that come out of the ChatGPT step, not the originals off the phone.</t>
+          <t>THUMBNAIL - the picture in the shop grid</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>This is a SEPARATE image, not one of the photos above. It is the single picture a customer</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>THE FIDDLY COLUMNS</t>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>sees while browsing, before they click in - so it is the one that sells the product.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>price, mrp, stock   Numbers only. 3950, never ₹3,950. mrp is the struck-through price — blank if no discount.</t>
-        </is>
-      </c>
+      <c r="A19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>category            Pick from the dropdown. Codes are on the 'Section codes' sheet.</t>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      thumbnail   krishna-flute-thumb.jpg</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>subCategory         Your own grouping, e.g. 'Brass Idols'. Spell it the same way every time.</t>
-        </is>
-      </c>
+      <c r="A21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>occasions           Any of: birthday, wedding, festival, everyday — semicolons between them.</t>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - It must be in the same folder as the photos.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>status              live = on the website now. draft = ready but held back. hidden = retired.</t>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Name it after the product with -thumb on the end, so it is obvious which is which.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>featured            yes puts it in the Shoppable Shorts rail. A handful only, or it stops being special.</t>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Roughly square works best. The grid crops to a square.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>description         A sentence or two. Commas are fine, Excel handles the quoting.</t>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - LEAVE IT BLANK and photo_1 is used instead. That is fine, and better than a bad</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr"/>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        thumbnail. Only fill it in when you have shot something for the grid specifically.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>BEFORE YOU SEND IT</t>
-        </is>
-      </c>
+      <c r="A27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">      • Sort by title — duplicates jump straight out.</t>
+          <t>FILENAME RULES - the part nobody can fix afterwards</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      • Check price and stock hold only numbers.</t>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - No spaces. Use hyphens.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      • Count the photo folder against the spreadsheet. The numbers should match.</t>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Every filename in the sheet must exist in the folder, spelled identically.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr"/>
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Krishna-Flute-01.JPG and krishna-flute-01.jpg are different files.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>SEND THE FIRST FIFTY FIRST.</t>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Send the images that come out of the ChatGPT step, not the originals off the phone.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>We will load them before the rest is finished. A format mistake caught on fifty rows costs an hour.</t>
-        </is>
-      </c>
+      <c r="A33" s="8" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Caught on a thousand, it costs a week.</t>
+          <t>THE FIDDLY COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>price, mrp, stock   Numbers only. 3950, never Rs 3,950. mrp is the struck-through price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>category            Pick from the dropdown. Codes are on the 'Section codes' sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>subCategory         Your own grouping, e.g. 'Brass Idols'. Spell it the same way every time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>occasions           Any of: birthday, wedding, festival, everyday - semicolons between them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>status              live = on the website now. draft = ready but held back. hidden = retired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>featured            yes puts it in the Shoppable Shorts rail. A handful only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>BEFORE YOU SEND IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Sort by title. Duplicates jump straight out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Check price and stock hold only numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Count the folder against the sheet: every photo_N and every thumbnail needs a file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>SEND THE FIRST FIFTY FIRST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>A format mistake caught on fifty rows costs an hour. Caught on a thousand, it costs a week.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Product videos: second in the gallery, playing by itself like Amazon
- New Videos collection (MP4/WebM/MOV, 50 MB cap), stored in the media
  volume under videos/, and a Video field on products. Migration adds the
  table and products.video_id; replayed up/down/up on an empty database.
- Product page: photo 1, then the video (muted, looping, inline, with
  controls; only loaded when its slide is shown), then the other photos.
  Its thumbnail carries a play badge; full screen plays it too.
- Google: the product's structured data lists the video (VideoObject).
- Bulk upload: new `video` column; picked videos go to the video library.
  Template and its instructions updated, with photo and video specs.
- Unused photos page now also finds unused videos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import/products-template.xlsx
+++ b/docs/import/products-template.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -485,26 +485,27 @@
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="48" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="28" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="40" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="28" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="40" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -548,102 +549,107 @@
           <t>thumbnail</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>mrp</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>subCategory</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>occasions</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>countryOfOrigin</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>genericName</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>netQuantity</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>dimensions</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>finish</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>monthYearOfImport</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>featured</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>shortCaption</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>shortSticker</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
@@ -678,96 +684,101 @@
           <t>krishna-flute-thumb.jpg</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>krishna-flute.mp4</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n">
         <v>3950</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>4500</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>pooja</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Brass Idols</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Brass Krishna standing with a flute, on a lotus base.</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>festival;wedding</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>Sri Balaji Handicrafts</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>Brass idol</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>1 piece</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>9 x 4 x 3 in</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>850 g</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>Antique brass</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>09/2026</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Y2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Z2" s="4" t="inlineStr">
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>The one everyone asks for</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="inlineStr">
+      <c r="AB2" s="4" t="inlineStr">
         <is>
           <t>Bestseller</t>
         </is>
       </c>
-      <c r="AB2" s="4" t="n"/>
+      <c r="AC2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -790,98 +801,99 @@
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n">
         <v>1299</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>1799</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>bags</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Slings &amp; Crossbody</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Compact tan sling with an adjustable strap and two zip pockets.</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>birthday;everyday</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>Hidesign Leathers</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>Sling bag</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>1 piece</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
+      <c r="U3" s="4" t="inlineStr">
         <is>
           <t>10 x 7 x 3 in</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="V3" s="4" t="inlineStr">
         <is>
           <t>420 g</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
+      <c r="W3" s="4" t="inlineStr">
         <is>
           <t>Genuine leather</t>
         </is>
       </c>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr">
         <is>
           <t>08/2026</t>
         </is>
       </c>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Y3" s="4" t="inlineStr">
+      <c r="Z3" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="4" t="n"/>
       <c r="AB3" s="4" t="n"/>
+      <c r="AC3" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="L2:L5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="One of the eight section codes - see the 'Section codes' sheet." promptTitle="Pick from the list" prompt="One of the eight section codes - see the 'Section codes' sheet." type="list">
+    <dataValidation sqref="M2:M5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="One of the eight section codes - see the 'Section codes' sheet." promptTitle="Pick from the list" prompt="One of the eight section codes - see the 'Section codes' sheet." type="list">
       <formula1>"decor,pooja,fashion,bags,shoes,watches,gifting,lifestyle"</formula1>
     </dataValidation>
-    <dataValidation sqref="X2:X5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="live = on the website. draft = held back. hidden = retired." promptTitle="Pick from the list" prompt="live = on the website. draft = held back. hidden = retired." type="list">
+    <dataValidation sqref="Y2:Y5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="live = on the website. draft = held back. hidden = retired." promptTitle="Pick from the list" prompt="live = on the website. draft = held back. hidden = retired." type="list">
       <formula1>"live,draft,hidden"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="yes puts it in the Shoppable Shorts rail. Keep this to a handful." promptTitle="Pick from the list" prompt="yes puts it in the Shoppable Shorts rail. Keep this to a handful." type="list">
+    <dataValidation sqref="Z2:Z5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid value" error="yes puts it in the Shoppable Shorts rail. Keep this to a handful." promptTitle="Pick from the list" prompt="yes puts it in the Shoppable Shorts rail. Keep this to a handful." type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1021,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -1120,36 +1132,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - 1600 x 2000 pixels (portrait, 4:5), JPG, under 1 MB each.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - photo_1 must be clean: no price, no text. Sizes and prices go on the last photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>THUMBNAIL - the picture in the shop grid</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>A SEPARATE image, not one of the photos above. It is the one picture a customer sees</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>while browsing, before they click in - so it is the one that sells the product.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      thumbnail   krishna-flute-thumb.jpg</t>
+          <t>while browsing, before they click in - so it is the one that sells the product.</t>
         </is>
       </c>
     </row>
@@ -1159,171 +1175,232 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - It goes in the same folder as the photos.</t>
+          <t xml:space="preserve">      thumbnail   krishna-flute-thumb.jpg</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - Name it after the product with -thumb on the end.</t>
-        </is>
-      </c>
+      <c r="A25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Roughly square works best. The grid crops to a square.</t>
+          <t xml:space="preserve">      - It goes in the same folder as the photos.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">      - Name it after the product with -thumb on the end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - 1600 x 2000 pixels, like the photos. The grid shows it at 4:5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">      - LEAVE IT BLANK and photo_1 is used instead. That is fine.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>FILENAME RULES - the part nobody can fix afterwards</t>
-        </is>
-      </c>
-    </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - No spaces. Use hyphens.</t>
-        </is>
-      </c>
+      <c r="A30" s="8" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - Every filename in the sheet must be in the folder, spelled exactly the same.</t>
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>VIDEO - optional, one per product</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Krishna-Flute-01.JPG and krishna-flute-01.jpg are different files.</t>
+          <t>Shown second on the product page, right after photo_1, and plays by itself (silent).</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - Send the images that come out of the ChatGPT step, not the originals off the phone.</t>
-        </is>
-      </c>
+      <c r="A33" s="8" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr"/>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      video   krishna-flute.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>THE FIDDLY COLUMNS</t>
-        </is>
-      </c>
+      <c r="A35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>price, mrp, stock   Numbers only. 3950, never Rs 3,950. mrp is the struck-through price.</t>
+          <t xml:space="preserve">      - MP4, vertical 9:16 (1080 x 1920), 15 to 30 seconds, under 50 MB.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>category            Pick from the dropdown. Codes are on the 'Section codes' sheet.</t>
+          <t xml:space="preserve">      - Same folder as the photos. Name it after the product.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>subCategory         Your own grouping, e.g. 'Brass Idols'. Spell it the same way every time.</t>
+          <t xml:space="preserve">      - No price or text on it, and no songs from Instagram or other apps.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>occasions           Any of: birthday, wedding, festival, everyday - semicolons between them.</t>
-        </is>
-      </c>
+      <c r="A39" s="8" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>status              live = on the website now. draft = ready but held back. hidden = retired.</t>
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>FILENAME RULES - the part nobody can fix afterwards</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>featured            yes puts it in the Shoppable Shorts rail. A handful only.</t>
+          <t xml:space="preserve">      - No spaces. Use hyphens.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>slug                LEAVE BLANK. It is the product's web address, filled in automatically.</t>
+          <t xml:space="preserve">      - Every filename in the sheet must be in the folder, spelled exactly the same.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    Only filled for products that already exist, so their links keep working.</t>
+          <t xml:space="preserve">        Krishna-Flute-01.JPG and krishna-flute-01.jpg are different files.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr"/>
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Send the images that come out of the ChatGPT step, not the originals off the phone.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>UPLOADING THE SAME SHEET TWICE IS SAFE</t>
-        </is>
-      </c>
+      <c r="A45" s="8" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>A product that already exists is updated, not copied. So you can fix a price in the sheet</t>
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>THE FIDDLY COLUMNS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>and upload it again.</t>
+          <t>price, mrp, stock   Numbers only. 3950, never Rs 3,950. mrp is the struck-through price.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr"/>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>category            Pick from the dropdown. Codes are on the 'Section codes' sheet.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>SEND THE FIRST FIFTY FIRST.</t>
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>subCategory         Your own grouping, e.g. 'Brass Idols'. Spell it the same way every time.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>occasions           Any of: birthday, wedding, festival, everyday - semicolons between them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>status              live = on the website now. draft = ready but held back. hidden = retired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>featured            yes puts it in the Shoppable Shorts rail. A handful only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>slug                LEAVE BLANK. It is the product's web address, filled in automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    Only filled for products that already exist, so their links keep working.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>UPLOADING THE SAME SHEET TWICE IS SAFE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>A product that already exists is updated, not copied. So you can fix a price in the sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>and upload it again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>SEND THE FIRST FIFTY FIRST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>A mistake caught on fifty rows costs an hour. Caught on a thousand, it costs a week.</t>
         </is>

</xml_diff>